<commit_message>
fluxo de credenciamento em imagem e inclusão de fabricantes / Publisher 3.0.1
</commit_message>
<xml_diff>
--- a/output/CodeSystem-BRFabricantePNI.xlsx
+++ b/output/CodeSystem-BRFabricantePNI.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="335">
   <si>
     <t>Property</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Fabricante do Imunobiológico (CodeSystem)</t>
+    <t>Fabricante do Imunobiológico</t>
   </si>
   <si>
     <t>Status</t>
@@ -991,6 +991,33 @@
   </si>
   <si>
     <t>LIBBS FARMACEUTICA LTDA.</t>
+  </si>
+  <si>
+    <t>47574</t>
+  </si>
+  <si>
+    <t>SANOFI-WIN</t>
+  </si>
+  <si>
+    <t>SANOFI WINTHROP INDUSTRIE</t>
+  </si>
+  <si>
+    <t>30426</t>
+  </si>
+  <si>
+    <t>FARMARIN</t>
+  </si>
+  <si>
+    <t>FARMARIN INDUSTRIA E COMERCIO LTDA.</t>
+  </si>
+  <si>
+    <t>30425</t>
+  </si>
+  <si>
+    <t>SAMTEC</t>
+  </si>
+  <si>
+    <t>SAMTEC BIOTECNOLOGIA LTDA</t>
   </si>
 </sst>
 </file>
@@ -1298,7 +1325,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2673,6 +2700,48 @@
         <v>325</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B99" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="C99" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="D99" t="s" s="2">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B100" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="C100" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="D100" t="s" s="2">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B101" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="C101" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="D101" t="s" s="2">
+        <v>334</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>